<commit_message>
docs: add product_name/channel_name display labels, unify basis gloss
Add `product_name`/`channel_name` columns to the segments sheet of the
sample basis workbooks (order: `product_code`, `product_name`,
`channel_code`, `channel_name`). These are report-side display labels the
reader ignores for matching -- the code/name pairing, mirroring
`coverage_code`/`coverage_name`.

Also unify the 산출기초 gloss to (가정), fix the two tree labels that
mislabelled basis.xlsx as 계리적 가정, and correct the column-value naming
table in design-decisions (`product_code`/`channel_code`, `TERM_LIFE_A`,
`coverage_code` casing, a `*_name` display-label row).
</commit_message>
<xml_diff>
--- a/src/fastcashflow/sample_data/sample_basis.xlsx
+++ b/src/fastcashflow/sample_data/sample_basis.xlsx
@@ -821,7 +821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -832,60 +832,70 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>product_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>channel_code</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>mortality_table</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>lapse_table</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>waiver_table</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>discount_table</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>inflation_table</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ra_confidence</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>mortality_cv</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>morbidity_cv</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>state_model</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>surrender_value_table</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>expense_table</t>
         </is>
@@ -897,41 +907,41 @@
           <t>defaults</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>MORTALITY_STD</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>WAIVER_STD</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>DISCOUNT_STD</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>INFL_BASE</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>0.75</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>0.1</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>0.12</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>WAIVER</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>SURRENDER_STD</t>
         </is>
@@ -945,15 +955,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>정기보험</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>FC</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>전속설계사</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>LAPSE_FC</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>EXP_TE_FC</t>
         </is>
@@ -967,15 +987,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>정기보험</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>GA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>법인대리점</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>LAPSE_GA</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>EXP_TE_GA</t>
         </is>
@@ -989,15 +1019,25 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>건강보험</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>FC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>전속설계사</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>LAPSE_FC</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>EXP_HE_FC</t>
         </is>
@@ -1011,15 +1051,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>건강보험</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>GA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>법인대리점</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>LAPSE_GA</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>EXP_HE_GA</t>
         </is>
@@ -1033,15 +1083,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>건강보험</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>텔레마케팅</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>LAPSE_GA</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>EXP_HE_TM</t>
         </is>
@@ -1055,15 +1115,25 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>종신보험</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>FC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>전속설계사</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>LAPSE_FC</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>EXP_WH_FC</t>
         </is>
@@ -1077,15 +1147,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>종신보험</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>GA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>법인대리점</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>LAPSE_GA</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>EXP_WH_GA</t>
         </is>

</xml_diff>